<commit_message>
fix the calcul of width cell in EMU
</commit_message>
<xml_diff>
--- a/test/templates/test-insert-images.xlsx
+++ b/test/templates/test-insert-images.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\surveaexcel\NEWER\jduxlsx\test\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jd2701\Documents\PROJECTS\SURVEA\XLSX-TEMPLATE\test\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C48689D8-E58F-42D8-BE1D-08AFC4911241}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89EF7A40-26B1-4B71-B502-F840CAD39936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="init_rels" sheetId="5" r:id="rId1"/>
     <sheet name="multi_test" sheetId="3" r:id="rId2"/>
     <sheet name="more_than_100" sheetId="6" r:id="rId3"/>
     <sheet name="breaking_image" sheetId="7" r:id="rId4"/>
+    <sheet name="width_height" sheetId="8" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="10">
   <si>
     <t>${image:imgB64}</t>
   </si>
@@ -52,6 +53,12 @@
   </si>
   <si>
     <t>${test}</t>
+  </si>
+  <si>
+    <t>${image:large}</t>
+  </si>
+  <si>
+    <t>Test width and height insert image in merge cells</t>
   </si>
 </sst>
 </file>
@@ -551,6 +558,9 @@
       <c r="U12" s="4"/>
     </row>
     <row r="13" spans="2:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="5" t="s">
+        <v>8</v>
+      </c>
       <c r="L13" s="4" t="s">
         <v>2</v>
       </c>
@@ -566,6 +576,7 @@
       <c r="U13" s="4"/>
     </row>
     <row r="14" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G14" s="5"/>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
       <c r="N14" s="3"/>
@@ -735,7 +746,8 @@
       <c r="U32" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="G13:G14"/>
     <mergeCell ref="I20:P22"/>
     <mergeCell ref="O4:P6"/>
     <mergeCell ref="O13:Q15"/>
@@ -788,4 +800,84 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FFA5C92-8E4F-4BFA-B478-52EB53B56525}">
+  <dimension ref="B1:I29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="5"/>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="5"/>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+    </row>
+    <row r="23" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="28" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F28" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+    </row>
+    <row r="29" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="C6:D12"/>
+    <mergeCell ref="F28:I29"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>